<commit_message>
drafting data skills s2
</commit_message>
<xml_diff>
--- a/skills/data/distributions_data.xlsx
+++ b/skills/data/distributions_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\non-od\KIND-training\skills\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1EFDD0A-69D2-4374-B0E0-C45DAC9FDA22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B5730B8-2043-4BCD-A0B7-0331F41B574E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{324A16CE-DABE-481D-940B-677BF89F85FD}"/>
+    <workbookView xWindow="57630" yWindow="32205" windowWidth="29040" windowHeight="17520" xr2:uid="{324A16CE-DABE-481D-940B-677BF89F85FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -962,9 +962,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0896856D-F1CF-45C2-AD34-D79B140184F1}">
   <dimension ref="A1:F323"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -984,7 +984,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1004,7 +1004,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1024,7 +1024,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1044,7 +1044,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1064,7 +1064,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1084,7 +1084,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1104,7 +1104,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1124,7 +1124,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1164,7 +1164,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1184,7 +1184,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1224,7 +1224,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1244,7 +1244,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1264,7 +1264,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1284,7 +1284,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1344,7 +1344,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1364,7 +1364,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1384,7 +1384,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1404,7 +1404,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1444,7 +1444,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1464,7 +1464,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1504,7 +1504,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1524,7 +1524,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1544,7 +1544,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1584,7 +1584,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1624,7 +1624,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1644,7 +1644,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1664,7 +1664,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1684,7 +1684,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1704,7 +1704,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1724,7 +1724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1744,7 +1744,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1764,7 +1764,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1844,7 +1844,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1864,7 +1864,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1884,7 +1884,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1904,7 +1904,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1964,7 +1964,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1984,7 +1984,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2004,7 +2004,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2044,7 +2044,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2064,7 +2064,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2084,7 +2084,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2144,7 +2144,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2184,7 +2184,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2224,7 +2224,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2264,7 +2264,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2304,7 +2304,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2318,13 +2318,13 @@
         <v>7</v>
       </c>
       <c r="E68">
-        <v>1021123123123</v>
+        <v>1021</v>
       </c>
       <c r="F68" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2364,7 +2364,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2384,7 +2384,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2444,7 +2444,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2484,7 +2484,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2504,7 +2504,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2524,7 +2524,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2544,7 +2544,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2604,7 +2604,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2684,7 +2684,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2704,7 +2704,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2804,7 +2804,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2844,7 +2844,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>94</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>95</v>
       </c>
@@ -2884,7 +2884,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>96</v>
       </c>
@@ -2904,7 +2904,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>97</v>
       </c>
@@ -2924,7 +2924,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>98</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>99</v>
       </c>
@@ -2964,7 +2964,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>100</v>
       </c>
@@ -2984,7 +2984,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>101</v>
       </c>
@@ -3004,7 +3004,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>102</v>
       </c>
@@ -3024,7 +3024,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>103</v>
       </c>
@@ -3044,7 +3044,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>104</v>
       </c>
@@ -3064,7 +3064,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>105</v>
       </c>
@@ -3084,7 +3084,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>106</v>
       </c>
@@ -3104,7 +3104,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>107</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>108</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>109</v>
       </c>
@@ -3164,7 +3164,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>110</v>
       </c>
@@ -3184,7 +3184,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>111</v>
       </c>
@@ -3204,7 +3204,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>112</v>
       </c>
@@ -3224,7 +3224,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>113</v>
       </c>
@@ -3244,7 +3244,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>114</v>
       </c>
@@ -3264,7 +3264,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>115</v>
       </c>
@@ -3284,7 +3284,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>116</v>
       </c>
@@ -3304,7 +3304,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>117</v>
       </c>
@@ -3324,7 +3324,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>118</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>119</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>120</v>
       </c>
@@ -3384,7 +3384,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>121</v>
       </c>
@@ -3404,7 +3404,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>122</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>123</v>
       </c>
@@ -3444,7 +3444,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>124</v>
       </c>
@@ -3464,7 +3464,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>125</v>
       </c>
@@ -3484,7 +3484,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>126</v>
       </c>
@@ -3504,7 +3504,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>127</v>
       </c>
@@ -3524,7 +3524,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>128</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>129</v>
       </c>
@@ -3564,7 +3564,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>130</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>131</v>
       </c>
@@ -3604,7 +3604,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>132</v>
       </c>
@@ -3624,7 +3624,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>133</v>
       </c>
@@ -3644,7 +3644,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>134</v>
       </c>
@@ -3664,7 +3664,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>135</v>
       </c>
@@ -3684,7 +3684,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>136</v>
       </c>
@@ -3704,7 +3704,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>137</v>
       </c>
@@ -3724,7 +3724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>138</v>
       </c>
@@ -3744,7 +3744,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>139</v>
       </c>
@@ -3764,7 +3764,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>140</v>
       </c>
@@ -3784,7 +3784,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>141</v>
       </c>
@@ -3804,7 +3804,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>142</v>
       </c>
@@ -3824,7 +3824,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>143</v>
       </c>
@@ -3844,7 +3844,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>144</v>
       </c>
@@ -3864,7 +3864,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>145</v>
       </c>
@@ -3884,7 +3884,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>146</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>147</v>
       </c>
@@ -3924,7 +3924,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>148</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>149</v>
       </c>
@@ -3964,7 +3964,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>150</v>
       </c>
@@ -3984,7 +3984,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>151</v>
       </c>
@@ -4004,7 +4004,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>152</v>
       </c>
@@ -4024,7 +4024,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>153</v>
       </c>
@@ -4044,7 +4044,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>154</v>
       </c>
@@ -4064,7 +4064,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>155</v>
       </c>
@@ -4084,7 +4084,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A157">
         <v>156</v>
       </c>
@@ -4104,7 +4104,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>157</v>
       </c>
@@ -4124,7 +4124,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>158</v>
       </c>
@@ -4144,7 +4144,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>159</v>
       </c>
@@ -4164,7 +4164,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A161">
         <v>160</v>
       </c>
@@ -4184,7 +4184,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A162">
         <v>161</v>
       </c>
@@ -4204,7 +4204,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A163">
         <v>162</v>
       </c>
@@ -4224,7 +4224,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A164">
         <v>163</v>
       </c>
@@ -4244,7 +4244,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A165">
         <v>164</v>
       </c>
@@ -4264,7 +4264,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A166">
         <v>165</v>
       </c>
@@ -4284,7 +4284,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A167">
         <v>166</v>
       </c>
@@ -4304,7 +4304,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A168">
         <v>167</v>
       </c>
@@ -4324,7 +4324,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A169">
         <v>168</v>
       </c>
@@ -4344,7 +4344,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A170">
         <v>169</v>
       </c>
@@ -4364,7 +4364,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A171">
         <v>170</v>
       </c>
@@ -4384,7 +4384,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A172">
         <v>171</v>
       </c>
@@ -4404,7 +4404,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A173">
         <v>172</v>
       </c>
@@ -4424,7 +4424,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A174">
         <v>173</v>
       </c>
@@ -4444,7 +4444,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A175">
         <v>174</v>
       </c>
@@ -4464,7 +4464,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A176">
         <v>175</v>
       </c>
@@ -4484,7 +4484,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A177">
         <v>176</v>
       </c>
@@ -4504,7 +4504,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A178">
         <v>177</v>
       </c>
@@ -4524,7 +4524,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A179">
         <v>178</v>
       </c>
@@ -4544,7 +4544,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A180">
         <v>179</v>
       </c>
@@ -4564,7 +4564,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A181">
         <v>180</v>
       </c>
@@ -4584,7 +4584,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A182">
         <v>181</v>
       </c>
@@ -4604,7 +4604,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A183">
         <v>182</v>
       </c>
@@ -4624,7 +4624,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A184">
         <v>183</v>
       </c>
@@ -4644,7 +4644,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A185">
         <v>184</v>
       </c>
@@ -4664,7 +4664,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A186">
         <v>185</v>
       </c>
@@ -4684,7 +4684,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A187">
         <v>186</v>
       </c>
@@ -4704,7 +4704,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A188">
         <v>187</v>
       </c>
@@ -4724,7 +4724,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A189">
         <v>188</v>
       </c>
@@ -4744,7 +4744,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A190">
         <v>189</v>
       </c>
@@ -4764,7 +4764,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A191">
         <v>190</v>
       </c>
@@ -4784,7 +4784,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A192">
         <v>191</v>
       </c>
@@ -4804,7 +4804,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A193">
         <v>192</v>
       </c>
@@ -4824,7 +4824,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A194">
         <v>193</v>
       </c>
@@ -4844,7 +4844,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A195">
         <v>194</v>
       </c>
@@ -4864,7 +4864,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A196">
         <v>195</v>
       </c>
@@ -4884,7 +4884,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A197">
         <v>196</v>
       </c>
@@ -4904,7 +4904,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A198">
         <v>197</v>
       </c>
@@ -4924,7 +4924,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A199">
         <v>198</v>
       </c>
@@ -4944,7 +4944,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A200">
         <v>199</v>
       </c>
@@ -4964,7 +4964,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A201">
         <v>200</v>
       </c>
@@ -4984,7 +4984,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A202">
         <v>201</v>
       </c>
@@ -5004,7 +5004,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A203">
         <v>202</v>
       </c>
@@ -5024,7 +5024,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A204">
         <v>203</v>
       </c>
@@ -5044,7 +5044,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A205">
         <v>204</v>
       </c>
@@ -5064,7 +5064,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A206">
         <v>205</v>
       </c>
@@ -5084,7 +5084,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A207">
         <v>206</v>
       </c>
@@ -5104,7 +5104,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A208">
         <v>207</v>
       </c>
@@ -5124,7 +5124,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A209">
         <v>208</v>
       </c>
@@ -5144,7 +5144,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A210">
         <v>209</v>
       </c>
@@ -5164,7 +5164,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A211">
         <v>210</v>
       </c>
@@ -5184,7 +5184,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A212">
         <v>211</v>
       </c>
@@ -5204,7 +5204,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A213">
         <v>212</v>
       </c>
@@ -5224,7 +5224,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A214">
         <v>213</v>
       </c>
@@ -5244,7 +5244,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A215">
         <v>214</v>
       </c>
@@ -5264,7 +5264,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A216">
         <v>215</v>
       </c>
@@ -5284,7 +5284,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A217">
         <v>216</v>
       </c>
@@ -5304,7 +5304,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A218">
         <v>217</v>
       </c>
@@ -5324,7 +5324,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A219">
         <v>218</v>
       </c>
@@ -5344,7 +5344,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A220">
         <v>219</v>
       </c>
@@ -5364,7 +5364,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A221">
         <v>220</v>
       </c>
@@ -5384,7 +5384,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A222">
         <v>221</v>
       </c>
@@ -5404,7 +5404,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A223">
         <v>222</v>
       </c>
@@ -5424,7 +5424,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A224">
         <v>223</v>
       </c>
@@ -5444,7 +5444,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A225">
         <v>224</v>
       </c>
@@ -5464,7 +5464,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A226">
         <v>225</v>
       </c>
@@ -5484,7 +5484,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A227">
         <v>226</v>
       </c>
@@ -5504,7 +5504,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A228">
         <v>227</v>
       </c>
@@ -5524,7 +5524,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A229">
         <v>228</v>
       </c>
@@ -5544,7 +5544,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A230">
         <v>229</v>
       </c>
@@ -5564,7 +5564,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A231">
         <v>230</v>
       </c>
@@ -5584,7 +5584,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A232">
         <v>231</v>
       </c>
@@ -5604,7 +5604,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A233">
         <v>232</v>
       </c>
@@ -5624,7 +5624,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A234">
         <v>233</v>
       </c>
@@ -5644,7 +5644,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A235">
         <v>234</v>
       </c>
@@ -5664,7 +5664,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A236">
         <v>235</v>
       </c>
@@ -5684,7 +5684,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A237">
         <v>236</v>
       </c>
@@ -5704,7 +5704,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A238">
         <v>237</v>
       </c>
@@ -5724,7 +5724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A239">
         <v>238</v>
       </c>
@@ -5744,7 +5744,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A240">
         <v>239</v>
       </c>
@@ -5764,7 +5764,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A241">
         <v>240</v>
       </c>
@@ -5784,7 +5784,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A242">
         <v>241</v>
       </c>
@@ -5804,7 +5804,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A243">
         <v>242</v>
       </c>
@@ -5824,7 +5824,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A244">
         <v>243</v>
       </c>
@@ -5844,7 +5844,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A245">
         <v>244</v>
       </c>
@@ -5864,7 +5864,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A246">
         <v>245</v>
       </c>
@@ -5884,7 +5884,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A247">
         <v>246</v>
       </c>
@@ -5904,7 +5904,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A248">
         <v>247</v>
       </c>
@@ -5924,7 +5924,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A249">
         <v>248</v>
       </c>
@@ -5944,7 +5944,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A250">
         <v>249</v>
       </c>
@@ -5964,7 +5964,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A251">
         <v>250</v>
       </c>
@@ -5984,7 +5984,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A252">
         <v>251</v>
       </c>
@@ -6004,7 +6004,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A253">
         <v>252</v>
       </c>
@@ -6024,7 +6024,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A254">
         <v>253</v>
       </c>
@@ -6044,7 +6044,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A255">
         <v>254</v>
       </c>
@@ -6064,7 +6064,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A256">
         <v>255</v>
       </c>
@@ -6084,7 +6084,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A257">
         <v>256</v>
       </c>
@@ -6104,7 +6104,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A258">
         <v>257</v>
       </c>
@@ -6124,7 +6124,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A259">
         <v>258</v>
       </c>
@@ -6144,7 +6144,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A260">
         <v>259</v>
       </c>
@@ -6164,7 +6164,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A261">
         <v>260</v>
       </c>
@@ -6184,7 +6184,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A262">
         <v>261</v>
       </c>
@@ -6204,7 +6204,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A263">
         <v>262</v>
       </c>
@@ -6224,7 +6224,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A264">
         <v>263</v>
       </c>
@@ -6244,7 +6244,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A265">
         <v>264</v>
       </c>
@@ -6264,7 +6264,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A266">
         <v>265</v>
       </c>
@@ -6284,7 +6284,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A267">
         <v>266</v>
       </c>
@@ -6304,7 +6304,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A268">
         <v>267</v>
       </c>
@@ -6324,7 +6324,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A269">
         <v>268</v>
       </c>
@@ -6344,7 +6344,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A270">
         <v>269</v>
       </c>
@@ -6364,7 +6364,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A271">
         <v>270</v>
       </c>
@@ -6384,7 +6384,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A272">
         <v>271</v>
       </c>
@@ -6404,7 +6404,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A273">
         <v>272</v>
       </c>
@@ -6424,7 +6424,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A274">
         <v>273</v>
       </c>
@@ -6444,7 +6444,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="275" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A275">
         <v>274</v>
       </c>
@@ -6464,7 +6464,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A276">
         <v>275</v>
       </c>
@@ -6484,7 +6484,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A277">
         <v>276</v>
       </c>
@@ -6504,7 +6504,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A278">
         <v>277</v>
       </c>
@@ -6524,7 +6524,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A279">
         <v>278</v>
       </c>
@@ -6544,7 +6544,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A280">
         <v>279</v>
       </c>
@@ -6564,7 +6564,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A281">
         <v>280</v>
       </c>
@@ -6584,7 +6584,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A282">
         <v>281</v>
       </c>
@@ -6604,7 +6604,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="283" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A283">
         <v>282</v>
       </c>
@@ -6624,7 +6624,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A284">
         <v>283</v>
       </c>
@@ -6644,7 +6644,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="285" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A285">
         <v>284</v>
       </c>
@@ -6664,7 +6664,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="286" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A286">
         <v>285</v>
       </c>
@@ -6684,7 +6684,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="287" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A287">
         <v>286</v>
       </c>
@@ -6704,7 +6704,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="288" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A288">
         <v>287</v>
       </c>
@@ -6724,7 +6724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A289">
         <v>288</v>
       </c>
@@ -6744,7 +6744,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A290">
         <v>289</v>
       </c>
@@ -6764,7 +6764,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="291" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A291">
         <v>290</v>
       </c>
@@ -6784,7 +6784,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="292" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A292">
         <v>291</v>
       </c>
@@ -6804,7 +6804,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="293" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A293">
         <v>292</v>
       </c>
@@ -6824,7 +6824,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A294">
         <v>293</v>
       </c>
@@ -6844,7 +6844,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="295" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A295">
         <v>294</v>
       </c>
@@ -6864,7 +6864,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="296" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A296">
         <v>295</v>
       </c>
@@ -6884,7 +6884,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="297" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A297">
         <v>296</v>
       </c>
@@ -6904,7 +6904,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="298" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A298">
         <v>297</v>
       </c>
@@ -6924,7 +6924,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="299" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A299">
         <v>298</v>
       </c>
@@ -6944,7 +6944,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A300">
         <v>299</v>
       </c>
@@ -6964,7 +6964,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="301" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A301">
         <v>300</v>
       </c>
@@ -6984,7 +6984,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="302" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A302">
         <v>301</v>
       </c>
@@ -7004,7 +7004,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="303" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A303">
         <v>302</v>
       </c>
@@ -7024,7 +7024,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="304" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A304">
         <v>303</v>
       </c>
@@ -7044,7 +7044,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="305" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A305">
         <v>304</v>
       </c>
@@ -7064,7 +7064,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="306" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A306">
         <v>305</v>
       </c>
@@ -7084,7 +7084,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A307">
         <v>306</v>
       </c>
@@ -7104,7 +7104,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="308" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A308">
         <v>307</v>
       </c>
@@ -7124,7 +7124,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="309" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A309">
         <v>308</v>
       </c>
@@ -7144,7 +7144,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A310">
         <v>309</v>
       </c>
@@ -7164,7 +7164,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="311" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A311">
         <v>310</v>
       </c>
@@ -7184,7 +7184,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="312" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A312">
         <v>311</v>
       </c>
@@ -7204,7 +7204,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="313" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A313">
         <v>312</v>
       </c>
@@ -7224,7 +7224,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="314" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A314">
         <v>313</v>
       </c>
@@ -7244,7 +7244,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="315" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A315">
         <v>314</v>
       </c>
@@ -7264,7 +7264,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="316" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A316">
         <v>315</v>
       </c>
@@ -7284,7 +7284,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="317" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A317">
         <v>316</v>
       </c>
@@ -7304,7 +7304,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="318" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A318">
         <v>317</v>
       </c>
@@ -7324,7 +7324,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="319" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A319">
         <v>318</v>
       </c>
@@ -7344,7 +7344,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="320" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A320">
         <v>319</v>
       </c>
@@ -7364,7 +7364,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A321">
         <v>320</v>
       </c>
@@ -7384,7 +7384,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="322" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A322">
         <v>321</v>
       </c>
@@ -7404,7 +7404,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="323" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A323">
         <v>322</v>
       </c>

</xml_diff>